<commit_message>
ATLAS 0.6.0: generazione delle schede Arcadia in Excel, import delle funzioni SA-2, ADR con decisione della DA
- Progetto > Genera: «Schede Arcadia» genera SA-1…SA-7 e le ADR in Excel dal modello, secondo le impostazioni
  salvate con il progetto («Impostazioni…»); template SA generati dalle schede (scripts/make_sa_templates.py)
- Import e re-import del catalogo SA-2 dei team, dalla scheda di una funzione e dal menu di SA-2
- ADR: membro proponente, sezione «Decisione della DA», stati In revisione DA e Revisionato DA, riallocazione di
  più clausole della stessa sezione, ADR inerenti nelle schede di dominio e funzione, lista ordinabile
- Barre di caricamento e aperture più rapide del report di copertura e del catalogo SRS
- Correzioni: dominio ereditato dalla sezione, clausole nella vista SA-2, spunte delle verifiche

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Templates/Template_SA-4_Requisiti_derivati.xlsx
+++ b/Templates/Template_SA-4_Requisiti_derivati.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SA-4" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'SA-4'!$A$1:$G$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'SA-4'!$A$1:$H$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -96,7 +96,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -118,11 +118,55 @@
         <color rgb="008EA9DB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="008EA9DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="008EA9DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="008EA9DB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="008EA9DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="008EA9DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="008EA9DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="008EA9DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="008EA9DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -145,7 +189,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -161,6 +205,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,16 +571,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="54" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -545,35 +591,35 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="39" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Template ARCADIA per i team di sviluppo · v1.0 · 28/09/2026 · Baseline delle specifiche: SUBSET-026 v3.6.0 (B3R2) · Chi compila: team del dominio · Livello: SA · Ordine di compilazione: 3 (insieme a SA-3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
+          <t>Template ARCADIA per i team di sviluppo · v1.1 · 30/10/2026 · Baseline delle specifiche: SUBSET-026 v3.6.0 (B3R2) · Chi compila: team del dominio · Livello: SA · Ordine di compilazione: 3 (insieme a SA-3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Scopo. Scomporre una voce che assegna obblighi a domini diversi in requisiti atomici, uno per dominio (Fase B6).</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="39" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Come si compila. Schema 1: più eventi convergono su una decisione; schema 2: la procedura (DF08) chiede un'azione al dominio proprietario; schema 3: più richieste arbitrate da un solo dominio. La voce madre è coperta quando lo sono tutti i derivati.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="17" customHeight="1">
+          <t>Come si compila. Schema 1: più eventi convergono su una decisione; schema 2: una procedura chiede un'azione al dominio che ne è responsabile; schema 3: più richieste arbitrate da un solo dominio. La voce madre è coperta quando lo sono tutti i derivati. In ATLAS è la scheda del requisito derivato (SA-4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Legenda: le celle bianche vanno compilate; il testo grigio in corsivo è guida o esempio del template e va sostituito. Le celle «Stato» e le colonne a valori fissi propongono un elenco a tendina.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Template</t>
@@ -594,17 +640,18 @@
           <t>es. T5 · DF07, DF08</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Versione</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>es. 0.1</t>
         </is>
       </c>
-      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="8" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -612,26 +659,27 @@
           <t>Autore</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr"/>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Revisore</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>gg/mm/aaaa</t>
         </is>
       </c>
-      <c r="G8" s="8" t="n"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
+      <c r="H8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Stato</t>
@@ -652,15 +700,16 @@
           <t>SUBSET-026 v3.6.0</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Rif. Capella / DOORS</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr"/>
-      <c r="G9" s="8" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="8" t="n"/>
+    </row>
+    <row r="11" ht="41" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
           <t>ID derivato</t>
@@ -668,36 +717,41 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
+          <t>Nome sintetico</t>
+        </is>
+      </c>
+      <c r="C11" s="9" t="inlineStr">
+        <is>
           <t>Voce madre</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Obbligo (una frase)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Funzione</t>
-        </is>
-      </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
+          <t>Funzione logica</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
           <t>Dominio</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Schema B6</t>
-        </is>
-      </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
+          <t>Motivazione della derivazione</t>
+        </is>
+      </c>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
           <t>Stato</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="54" customHeight="1">
       <c r="A12" s="10" t="inlineStr">
         <is>
           <t>5.11.2.2-A030-D1</t>
@@ -705,34 +759,41 @@
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
+          <t>Evento di report di posizione</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
           <t>5.11.2.2-A030</t>
         </is>
       </c>
-      <c r="C12" s="10" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>Il cambio di modo genera un evento di report di posizione</t>
         </is>
       </c>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>SF-DF02-11</t>
-        </is>
-      </c>
       <c r="E12" s="10" t="inlineStr">
         <is>
+          <t>LF-DF02-11-01</t>
+        </is>
+      </c>
+      <c r="F12" s="10" t="inlineStr">
+        <is>
           <t>DF02</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
+          <t>2 – Una procedura chiede un'azione al dominio che ne è responsabile</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
           <t>Proposto</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
+    <row r="13" ht="28" customHeight="1">
       <c r="A13" s="11" t="n"/>
       <c r="B13" s="11" t="n"/>
       <c r="C13" s="11" t="n"/>
@@ -740,8 +801,9 @@
       <c r="E13" s="11" t="n"/>
       <c r="F13" s="11" t="n"/>
       <c r="G13" s="11" t="n"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
+      <c r="H13" s="11" t="n"/>
+    </row>
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="11" t="n"/>
       <c r="B14" s="11" t="n"/>
       <c r="C14" s="11" t="n"/>
@@ -749,8 +811,9 @@
       <c r="E14" s="11" t="n"/>
       <c r="F14" s="11" t="n"/>
       <c r="G14" s="11" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
+      <c r="H14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="28" customHeight="1">
       <c r="A15" s="11" t="n"/>
       <c r="B15" s="11" t="n"/>
       <c r="C15" s="11" t="n"/>
@@ -758,8 +821,9 @@
       <c r="E15" s="11" t="n"/>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="11" t="n"/>
-    </row>
-    <row r="16" ht="20" customHeight="1">
+      <c r="H15" s="11" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="11" t="n"/>
       <c r="B16" s="11" t="n"/>
       <c r="C16" s="11" t="n"/>
@@ -767,8 +831,9 @@
       <c r="E16" s="11" t="n"/>
       <c r="F16" s="11" t="n"/>
       <c r="G16" s="11" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
+      <c r="H16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="11" t="n"/>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="11" t="n"/>
@@ -776,8 +841,9 @@
       <c r="E17" s="11" t="n"/>
       <c r="F17" s="11" t="n"/>
       <c r="G17" s="11" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
+      <c r="H17" s="11" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="11" t="n"/>
       <c r="B18" s="11" t="n"/>
       <c r="C18" s="11" t="n"/>
@@ -785,8 +851,9 @@
       <c r="E18" s="11" t="n"/>
       <c r="F18" s="11" t="n"/>
       <c r="G18" s="11" t="n"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
+      <c r="H18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="28" customHeight="1">
       <c r="A19" s="11" t="n"/>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
@@ -794,8 +861,9 @@
       <c r="E19" s="11" t="n"/>
       <c r="F19" s="11" t="n"/>
       <c r="G19" s="11" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
+      <c r="H19" s="11" t="n"/>
+    </row>
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="11" t="n"/>
       <c r="B20" s="11" t="n"/>
       <c r="C20" s="11" t="n"/>
@@ -803,8 +871,9 @@
       <c r="E20" s="11" t="n"/>
       <c r="F20" s="11" t="n"/>
       <c r="G20" s="11" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+      <c r="H20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="28" customHeight="1">
       <c r="A21" s="11" t="n"/>
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="11" t="n"/>
@@ -812,8 +881,9 @@
       <c r="E21" s="11" t="n"/>
       <c r="F21" s="11" t="n"/>
       <c r="G21" s="11" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
+      <c r="H21" s="11" t="n"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="11" t="n"/>
       <c r="B22" s="11" t="n"/>
       <c r="C22" s="11" t="n"/>
@@ -821,8 +891,9 @@
       <c r="E22" s="11" t="n"/>
       <c r="F22" s="11" t="n"/>
       <c r="G22" s="11" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
+      <c r="H22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="11" t="n"/>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="11" t="n"/>
@@ -830,8 +901,9 @@
       <c r="E23" s="11" t="n"/>
       <c r="F23" s="11" t="n"/>
       <c r="G23" s="11" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
+      <c r="H23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="11" t="n"/>
       <c r="B24" s="11" t="n"/>
       <c r="C24" s="11" t="n"/>
@@ -839,8 +911,9 @@
       <c r="E24" s="11" t="n"/>
       <c r="F24" s="11" t="n"/>
       <c r="G24" s="11" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
+      <c r="H24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="11" t="n"/>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
@@ -848,8 +921,9 @@
       <c r="E25" s="11" t="n"/>
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
+      <c r="H25" s="11" t="n"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="11" t="n"/>
       <c r="B26" s="11" t="n"/>
       <c r="C26" s="11" t="n"/>
@@ -857,8 +931,9 @@
       <c r="E26" s="11" t="n"/>
       <c r="F26" s="11" t="n"/>
       <c r="G26" s="11" t="n"/>
-    </row>
-    <row r="27" ht="20" customHeight="1">
+      <c r="H26" s="11" t="n"/>
+    </row>
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="11" t="n"/>
       <c r="B27" s="11" t="n"/>
       <c r="C27" s="11" t="n"/>
@@ -866,6 +941,7 @@
       <c r="E27" s="11" t="n"/>
       <c r="F27" s="11" t="n"/>
       <c r="G27" s="11" t="n"/>
+      <c r="H27" s="11" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="12" t="inlineStr">
@@ -874,7 +950,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="13" t="inlineStr">
         <is>
           <t>☐</t>
@@ -885,13 +961,14 @@
           <t>Ogni derivato ha un solo obbligo e un solo dominio</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="8" t="n"/>
-      <c r="G30" s="8" t="n"/>
-    </row>
-    <row r="31" ht="18" customHeight="1">
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
+      <c r="G30" s="14" t="n"/>
+      <c r="H30" s="8" t="n"/>
+    </row>
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="13" t="inlineStr">
         <is>
           <t>☐</t>
@@ -902,13 +979,14 @@
           <t>Il dominio assegnato è il proprietario del dato o dell'azione</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="8" t="n"/>
-      <c r="G31" s="8" t="n"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="8" t="n"/>
+    </row>
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
           <t>☐</t>
@@ -919,47 +997,133 @@
           <t>Nessun derivato crea un secondo produttore per un dato esistente</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="8" t="n"/>
-      <c r="G32" s="8" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="8" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B32:G32"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="A5:G5"/>
-    <mergeCell ref="F8:G8"/>
+  <mergeCells count="15">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B32:H32"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B31:H31"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="33">
     <dataValidation sqref="B9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Bozza,In revisione,Approvato"</formula1>
     </dataValidation>
-    <dataValidation sqref="F12:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1,2,3"</formula1>
-    </dataValidation>
-    <dataValidation sqref="A30 A31 A32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"☐,☑"</formula1>
+    <dataValidation sqref="G12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1 – Più eventi, anche da domini diversi, portano a un'unica decisione,2 – Una procedura chiede un'azione al dominio che ne è responsabile,3 – Più richieste, anche da domini diversi, sono decise da un solo dominio"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Proposto,Rivisto,Approvato"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 Informazione ad uso interno - Internal use information&amp;R&amp;8 &amp;P / &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>